<commit_message>
feat(loom): chart matplotlib bonito + drop Zelle wording (LATAM friendly)
- Chart Cashflow ahora es PNG matplotlib embebido (brand colors, area fill,
  bars verde/rojo para flujo neto, sin gridlines, fechas legibles)
- Sheet renombra "REPOSITORIO ZELLE" -> "REPOSITORIO DE PAGOS Y COBROS"
- Cheatsheet y walkthrough drop Zelle wording: "transferencia bancaria",
  "comprobante de pago", "captura del banco" para que LATAM (Mexico, Colombia,
  Peru, Argentina donde Zelle no existe) entienda
- Capturas mantienen logos BoA/Chase pero el discurso es generico

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/posts/demo-sheet-for-loom.xlsx
+++ b/posts/demo-sheet-for-loom.xlsx
@@ -567,158 +567,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Cashflow diario · Saldo acumulado</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Cashflow'!E5</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cashflow'!$B$6:$B$22</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cashflow'!$E$6:$E$22</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Cashflow'!F5</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cashflow'!$B$6:$B$22</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cashflow'!$F$6:$F$22</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Fecha</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-        <tickLblSkip val="2"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Monto USD</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -785,22 +633,25 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9360000" cy="3960000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="7810500" cy="3333750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -1120,7 +971,7 @@
     <row r="11" ht="42" customHeight="1">
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>REPOSITORIO ZELLE  ·  CONTROL FINANCIERO 360</t>
+          <t>REPOSITORIO DE PAGOS Y COBROS  ·  CONTROL FINANCIERO 360</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(loom): Cashflow horizontal + KPIs visual + colores IB
- Cashflow tab: layout horizontal (fechas como columnas, metricas como
  filas Ingresos/Gastos/Flujo/Saldo Acumulado) tipo dashboard ejecutivo.
  Total al final, saldo inicial referenciado arriba derecha.
- KPIs tab: rediseno con 4 secciones (Ingresos, Gastos, Operacion,
  Posicion de efectivo), hero "Flujo Neto" grande, leyenda de colores.
- Colores IB aplicados: AZUL=hardcoded input, NEGRO=formula misma hoja,
  VERDE=link cross-sheet (referencia a otra pestana).
- Cashflow chart matplotlib reposicionado debajo de la tabla.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/posts/demo-sheet-for-loom.xlsx
+++ b/posts/demo-sheet-for-loom.xlsx
@@ -21,13 +21,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0&quot; gandolas&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; cobros&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.00\%"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0;[Red]-&quot;$&quot;#,##0;&quot;&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.00\%"/>
+    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00;[Red]-&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="42">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,7 +79,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002563EB"/>
+      <color rgb="000070C0"/>
       <sz val="11"/>
     </font>
     <font>
@@ -86,7 +89,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4D2E"/>
+      <color rgb="001A1A1A"/>
       <sz val="36"/>
     </font>
     <font>
@@ -101,7 +104,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4D2E"/>
+      <color rgb="0000B050"/>
       <sz val="20"/>
     </font>
     <font>
@@ -111,7 +114,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00059669"/>
+      <color rgb="001A1A1A"/>
       <sz val="20"/>
     </font>
     <font>
@@ -156,26 +159,27 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002563EB"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="00166534"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="00991B1B"/>
+      <color rgb="000070C0"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4D2E"/>
-      <sz val="11"/>
+      <color rgb="0000B050"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00991B1B"/>
-      <sz val="11"/>
+      <color rgb="00C9A961"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="0000B050"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -184,16 +188,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00059669"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="001F4D2E"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00059669"/>
+      <color rgb="0000B050"/>
       <sz val="11"/>
     </font>
     <font>
@@ -201,25 +200,45 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="002563EB"/>
+      <color rgb="000070C0"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4D2E"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <color rgb="001A1A1A"/>
-      <sz val="11"/>
+      <color rgb="00C9A961"/>
+      <sz val="20"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002563EB"/>
-      <sz val="12"/>
+      <color rgb="0000B050"/>
+      <sz val="40"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4D2E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000B050"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -266,6 +285,31 @@
         <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B6914"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9A961"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -293,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -353,34 +397,34 @@
     <xf numFmtId="164" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -453,18 +497,46 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="164" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="29" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -472,25 +544,92 @@
     <xf numFmtId="164" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="36" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="38" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -631,12 +770,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7810500" cy="3333750"/>
+    <ext cx="9334500" cy="3619500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2883,19 +3022,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J23"/>
+  <dimension ref="B2:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="4" customWidth="1" min="7" max="7"/>
-    <col width="4" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="2" ht="38" customHeight="1">
@@ -2908,464 +3057,437 @@
     <row r="3">
       <c r="B3" s="56" t="inlineStr">
         <is>
-          <t>Movimientos consolidados por fecha. Ingresos / Gastos / Flujo / Saldo acumulado.</t>
-        </is>
-      </c>
-      <c r="I3" s="57" t="inlineStr">
+          <t>Movimientos consolidados por fecha. Filas: Ingresos / Gastos / Flujo Neto / Saldo Acumulado.</t>
+        </is>
+      </c>
+      <c r="R3" s="57" t="inlineStr">
         <is>
           <t>Saldo inicial (Dashboard!E5):</t>
         </is>
       </c>
-      <c r="J3" s="58">
+      <c r="U3" s="58">
         <f>Dashboard!E5</f>
         <v/>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Ingresos</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Gastos</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Flujo Neto</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>Saldo Acumulado</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-18</t>
-        </is>
-      </c>
-      <c r="C6" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-18")</f>
-        <v/>
-      </c>
-      <c r="D6" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-18")</f>
-        <v/>
-      </c>
-      <c r="E6" s="61">
-        <f>C6-D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="58">
-        <f>$J$3+E6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-19</t>
-        </is>
-      </c>
-      <c r="C7" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-19")</f>
-        <v/>
-      </c>
-      <c r="D7" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-19")</f>
-        <v/>
-      </c>
-      <c r="E7" s="61">
-        <f>C7-D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="58">
-        <f>F6+E7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="C8" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-20")</f>
-        <v/>
-      </c>
-      <c r="D8" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-20")</f>
-        <v/>
-      </c>
-      <c r="E8" s="61">
-        <f>C8-D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="58">
-        <f>F7+E8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-21</t>
-        </is>
-      </c>
-      <c r="C9" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-21")</f>
-        <v/>
-      </c>
-      <c r="D9" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-21")</f>
-        <v/>
-      </c>
-      <c r="E9" s="61">
-        <f>C9-D9</f>
-        <v/>
-      </c>
-      <c r="F9" s="58">
-        <f>F8+E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="C10" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-22")</f>
-        <v/>
-      </c>
-      <c r="D10" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-22")</f>
-        <v/>
-      </c>
-      <c r="E10" s="61">
-        <f>C10-D10</f>
-        <v/>
-      </c>
-      <c r="F10" s="58">
-        <f>F9+E10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="C11" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-23")</f>
-        <v/>
-      </c>
-      <c r="D11" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-23")</f>
-        <v/>
-      </c>
-      <c r="E11" s="61">
-        <f>C11-D11</f>
-        <v/>
-      </c>
-      <c r="F11" s="58">
-        <f>F10+E11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="C12" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-24")</f>
-        <v/>
-      </c>
-      <c r="D12" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-24")</f>
-        <v/>
-      </c>
-      <c r="E12" s="61">
-        <f>C12-D12</f>
-        <v/>
-      </c>
-      <c r="F12" s="58">
-        <f>F11+E12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-25</t>
-        </is>
-      </c>
-      <c r="C13" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-25")</f>
-        <v/>
-      </c>
-      <c r="D13" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-25")</f>
-        <v/>
-      </c>
-      <c r="E13" s="61">
-        <f>C13-D13</f>
-        <v/>
-      </c>
-      <c r="F13" s="58">
-        <f>F12+E13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="C14" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-26")</f>
-        <v/>
-      </c>
-      <c r="D14" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-26")</f>
-        <v/>
-      </c>
-      <c r="E14" s="61">
-        <f>C14-D14</f>
-        <v/>
-      </c>
-      <c r="F14" s="58">
-        <f>F13+E14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="C15" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-27")</f>
-        <v/>
-      </c>
-      <c r="D15" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-27")</f>
-        <v/>
-      </c>
-      <c r="E15" s="61">
-        <f>C15-D15</f>
-        <v/>
-      </c>
-      <c r="F15" s="58">
-        <f>F14+E15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C16" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-28")</f>
-        <v/>
-      </c>
-      <c r="D16" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-28")</f>
-        <v/>
-      </c>
-      <c r="E16" s="61">
-        <f>C16-D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="58">
-        <f>F15+E16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="C17" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-29")</f>
-        <v/>
-      </c>
-      <c r="D17" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-29")</f>
-        <v/>
-      </c>
-      <c r="E17" s="61">
-        <f>C17-D17</f>
-        <v/>
-      </c>
-      <c r="F17" s="58">
-        <f>F16+E17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="44" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C18" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-04-30")</f>
-        <v/>
-      </c>
-      <c r="D18" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-04-30")</f>
-        <v/>
-      </c>
-      <c r="E18" s="61">
-        <f>C18-D18</f>
-        <v/>
-      </c>
-      <c r="F18" s="58">
-        <f>F17+E18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="C19" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-05-01")</f>
-        <v/>
-      </c>
-      <c r="D19" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-05-01")</f>
-        <v/>
-      </c>
-      <c r="E19" s="61">
-        <f>C19-D19</f>
-        <v/>
-      </c>
-      <c r="F19" s="58">
-        <f>F18+E19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="44" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="C20" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-05-02")</f>
-        <v/>
-      </c>
-      <c r="D20" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-05-02")</f>
-        <v/>
-      </c>
-      <c r="E20" s="61">
-        <f>C20-D20</f>
-        <v/>
-      </c>
-      <c r="F20" s="58">
-        <f>F19+E20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="44" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="C21" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-05-03")</f>
-        <v/>
-      </c>
-      <c r="D21" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-05-03")</f>
-        <v/>
-      </c>
-      <c r="E21" s="61">
-        <f>C21-D21</f>
-        <v/>
-      </c>
-      <c r="F21" s="58">
-        <f>F20+E21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="44" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="C22" s="59">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in",Transacciones!B:B,"2026-05-04")</f>
-        <v/>
-      </c>
-      <c r="D22" s="60">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out",Transacciones!B:B,"2026-05-04")</f>
-        <v/>
-      </c>
-      <c r="E22" s="61">
-        <f>C22-D22</f>
-        <v/>
-      </c>
-      <c r="F22" s="58">
-        <f>F21+E22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="62" t="inlineStr">
-        <is>
-          <t>TOTAL PERIODO</t>
-        </is>
-      </c>
-      <c r="C23" s="63">
-        <f>SUM(C6:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="64">
-        <f>SUM(D6:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="65">
-        <f>C23-D23</f>
-        <v/>
-      </c>
-      <c r="F23" s="66">
-        <f>F22</f>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C5" s="59" t="inlineStr">
+        <is>
+          <t>18-Apr</t>
+        </is>
+      </c>
+      <c r="D5" s="59" t="inlineStr">
+        <is>
+          <t>19-Apr</t>
+        </is>
+      </c>
+      <c r="E5" s="59" t="inlineStr">
+        <is>
+          <t>20-Apr</t>
+        </is>
+      </c>
+      <c r="F5" s="59" t="inlineStr">
+        <is>
+          <t>21-Apr</t>
+        </is>
+      </c>
+      <c r="G5" s="59" t="inlineStr">
+        <is>
+          <t>22-Apr</t>
+        </is>
+      </c>
+      <c r="H5" s="59" t="inlineStr">
+        <is>
+          <t>23-Apr</t>
+        </is>
+      </c>
+      <c r="I5" s="59" t="inlineStr">
+        <is>
+          <t>24-Apr</t>
+        </is>
+      </c>
+      <c r="J5" s="59" t="inlineStr">
+        <is>
+          <t>25-Apr</t>
+        </is>
+      </c>
+      <c r="K5" s="59" t="inlineStr">
+        <is>
+          <t>26-Apr</t>
+        </is>
+      </c>
+      <c r="L5" s="59" t="inlineStr">
+        <is>
+          <t>27-Apr</t>
+        </is>
+      </c>
+      <c r="M5" s="59" t="inlineStr">
+        <is>
+          <t>28-Apr</t>
+        </is>
+      </c>
+      <c r="N5" s="59" t="inlineStr">
+        <is>
+          <t>29-Apr</t>
+        </is>
+      </c>
+      <c r="O5" s="59" t="inlineStr">
+        <is>
+          <t>30-Apr</t>
+        </is>
+      </c>
+      <c r="P5" s="59" t="inlineStr">
+        <is>
+          <t>01-May</t>
+        </is>
+      </c>
+      <c r="Q5" s="59" t="inlineStr">
+        <is>
+          <t>02-May</t>
+        </is>
+      </c>
+      <c r="R5" s="59" t="inlineStr">
+        <is>
+          <t>03-May</t>
+        </is>
+      </c>
+      <c r="S5" s="59" t="inlineStr">
+        <is>
+          <t>04-May</t>
+        </is>
+      </c>
+      <c r="T5" s="60" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="B6" s="61" t="inlineStr">
+        <is>
+          <t>INGRESOS</t>
+        </is>
+      </c>
+      <c r="C6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-18")</f>
+        <v/>
+      </c>
+      <c r="D6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-19")</f>
+        <v/>
+      </c>
+      <c r="E6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-20")</f>
+        <v/>
+      </c>
+      <c r="F6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-21")</f>
+        <v/>
+      </c>
+      <c r="G6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-22")</f>
+        <v/>
+      </c>
+      <c r="H6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-23")</f>
+        <v/>
+      </c>
+      <c r="I6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-24")</f>
+        <v/>
+      </c>
+      <c r="J6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-25")</f>
+        <v/>
+      </c>
+      <c r="K6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-26")</f>
+        <v/>
+      </c>
+      <c r="L6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-27")</f>
+        <v/>
+      </c>
+      <c r="M6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-28")</f>
+        <v/>
+      </c>
+      <c r="N6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-29")</f>
+        <v/>
+      </c>
+      <c r="O6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-04-30")</f>
+        <v/>
+      </c>
+      <c r="P6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-05-01")</f>
+        <v/>
+      </c>
+      <c r="Q6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-05-02")</f>
+        <v/>
+      </c>
+      <c r="R6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-05-03")</f>
+        <v/>
+      </c>
+      <c r="S6" s="62">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"in",Transacciones!$B:$B,"2026-05-04")</f>
+        <v/>
+      </c>
+      <c r="T6" s="63">
+        <f>SUM(C6:S6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="B7" s="64" t="inlineStr">
+        <is>
+          <t>GASTOS</t>
+        </is>
+      </c>
+      <c r="C7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-18")</f>
+        <v/>
+      </c>
+      <c r="D7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-19")</f>
+        <v/>
+      </c>
+      <c r="E7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-20")</f>
+        <v/>
+      </c>
+      <c r="F7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-21")</f>
+        <v/>
+      </c>
+      <c r="G7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-22")</f>
+        <v/>
+      </c>
+      <c r="H7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-23")</f>
+        <v/>
+      </c>
+      <c r="I7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-24")</f>
+        <v/>
+      </c>
+      <c r="J7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-25")</f>
+        <v/>
+      </c>
+      <c r="K7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-26")</f>
+        <v/>
+      </c>
+      <c r="L7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-27")</f>
+        <v/>
+      </c>
+      <c r="M7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-28")</f>
+        <v/>
+      </c>
+      <c r="N7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-29")</f>
+        <v/>
+      </c>
+      <c r="O7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-04-30")</f>
+        <v/>
+      </c>
+      <c r="P7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-05-01")</f>
+        <v/>
+      </c>
+      <c r="Q7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-05-02")</f>
+        <v/>
+      </c>
+      <c r="R7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-05-03")</f>
+        <v/>
+      </c>
+      <c r="S7" s="65">
+        <f>SUMIFS(Transacciones!$D:$D,Transacciones!$E:$E,"out",Transacciones!$B:$B,"2026-05-04")</f>
+        <v/>
+      </c>
+      <c r="T7" s="63">
+        <f>SUM(C7:S7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>FLUJO NETO</t>
+        </is>
+      </c>
+      <c r="C8" s="67">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="67">
+        <f>D6-D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="67">
+        <f>E6-E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="67">
+        <f>F6-F7</f>
+        <v/>
+      </c>
+      <c r="G8" s="67">
+        <f>G6-G7</f>
+        <v/>
+      </c>
+      <c r="H8" s="67">
+        <f>H6-H7</f>
+        <v/>
+      </c>
+      <c r="I8" s="67">
+        <f>I6-I7</f>
+        <v/>
+      </c>
+      <c r="J8" s="67">
+        <f>J6-J7</f>
+        <v/>
+      </c>
+      <c r="K8" s="67">
+        <f>K6-K7</f>
+        <v/>
+      </c>
+      <c r="L8" s="67">
+        <f>L6-L7</f>
+        <v/>
+      </c>
+      <c r="M8" s="67">
+        <f>M6-M7</f>
+        <v/>
+      </c>
+      <c r="N8" s="67">
+        <f>N6-N7</f>
+        <v/>
+      </c>
+      <c r="O8" s="67">
+        <f>O6-O7</f>
+        <v/>
+      </c>
+      <c r="P8" s="67">
+        <f>P6-P7</f>
+        <v/>
+      </c>
+      <c r="Q8" s="67">
+        <f>Q6-Q7</f>
+        <v/>
+      </c>
+      <c r="R8" s="67">
+        <f>R6-R7</f>
+        <v/>
+      </c>
+      <c r="S8" s="67">
+        <f>S6-S7</f>
+        <v/>
+      </c>
+      <c r="T8" s="63">
+        <f>T6-T7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="B9" s="68" t="inlineStr">
+        <is>
+          <t>SALDO ACUMULADO</t>
+        </is>
+      </c>
+      <c r="C9" s="69">
+        <f>$U$3+C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="69">
+        <f>C9+D8</f>
+        <v/>
+      </c>
+      <c r="E9" s="69">
+        <f>D9+E8</f>
+        <v/>
+      </c>
+      <c r="F9" s="69">
+        <f>E9+F8</f>
+        <v/>
+      </c>
+      <c r="G9" s="69">
+        <f>F9+G8</f>
+        <v/>
+      </c>
+      <c r="H9" s="69">
+        <f>G9+H8</f>
+        <v/>
+      </c>
+      <c r="I9" s="69">
+        <f>H9+I8</f>
+        <v/>
+      </c>
+      <c r="J9" s="69">
+        <f>I9+J8</f>
+        <v/>
+      </c>
+      <c r="K9" s="69">
+        <f>J9+K8</f>
+        <v/>
+      </c>
+      <c r="L9" s="69">
+        <f>K9+L8</f>
+        <v/>
+      </c>
+      <c r="M9" s="69">
+        <f>L9+M8</f>
+        <v/>
+      </c>
+      <c r="N9" s="69">
+        <f>M9+N8</f>
+        <v/>
+      </c>
+      <c r="O9" s="69">
+        <f>N9+O8</f>
+        <v/>
+      </c>
+      <c r="P9" s="69">
+        <f>O9+P8</f>
+        <v/>
+      </c>
+      <c r="Q9" s="69">
+        <f>P9+Q8</f>
+        <v/>
+      </c>
+      <c r="R9" s="69">
+        <f>Q9+R8</f>
+        <v/>
+      </c>
+      <c r="S9" s="69">
+        <f>R9+S8</f>
+        <v/>
+      </c>
+      <c r="T9" s="70">
+        <f>$U$3+T8</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B2:G2"/>
+  <mergeCells count="3">
+    <mergeCell ref="B2:U2"/>
+    <mergeCell ref="B3:Q3"/>
+    <mergeCell ref="R3:T3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3398,7 +3520,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="71" t="inlineStr">
         <is>
           <t>DEUDAS  ·  Por cobrar / Por pagar</t>
         </is>
@@ -3477,130 +3599,130 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="68" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>Luis Mendoza</t>
         </is>
       </c>
-      <c r="B4" s="68" t="inlineStr">
+      <c r="B4" s="72" t="inlineStr">
         <is>
           <t>Por Pagar</t>
         </is>
       </c>
-      <c r="C4" s="69" t="n">
+      <c r="C4" s="73" t="n">
         <v>40000</v>
       </c>
-      <c r="D4" s="68" t="inlineStr">
+      <c r="D4" s="72" t="inlineStr">
         <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n">
+      <c r="E4" s="74" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="68" t="n">
+      <c r="F4" s="72" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="71" t="n">
+      <c r="G4" s="75" t="n">
         <v>1600</v>
       </c>
-      <c r="H4" s="71" t="n">
+      <c r="H4" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="72" t="n">
+      <c r="I4" s="76" t="n">
         <v>40000</v>
       </c>
-      <c r="J4" s="68" t="inlineStr"/>
-      <c r="K4" s="68" t="inlineStr"/>
-      <c r="L4" s="68" t="inlineStr">
+      <c r="J4" s="72" t="inlineStr"/>
+      <c r="K4" s="72" t="inlineStr"/>
+      <c r="L4" s="72" t="inlineStr">
         <is>
           <t>Transferencia mensual</t>
         </is>
       </c>
-      <c r="M4" s="68" t="inlineStr">
+      <c r="M4" s="72" t="inlineStr">
         <is>
           <t>Sin vcto.</t>
         </is>
       </c>
-      <c r="N4" s="68" t="inlineStr">
+      <c r="N4" s="72" t="inlineStr">
         <is>
           <t>Prestamo dic 2025. Capital $40,000. Interes 4% mensual fijo $1,600. Solo se pagan intereses; capital intacto.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="68" t="inlineStr">
+      <c r="A5" s="72" t="inlineStr">
         <is>
           <t>Pedro Ramos</t>
         </is>
       </c>
-      <c r="B5" s="68" t="inlineStr">
+      <c r="B5" s="72" t="inlineStr">
         <is>
           <t>Por Pagar</t>
         </is>
       </c>
-      <c r="C5" s="69" t="n">
+      <c r="C5" s="73" t="n">
         <v>50000</v>
       </c>
-      <c r="D5" s="68" t="inlineStr">
+      <c r="D5" s="72" t="inlineStr">
         <is>
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="E5" s="70" t="n">
+      <c r="E5" s="74" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="68" t="n">
+      <c r="F5" s="72" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="71" t="n">
+      <c r="G5" s="75" t="n">
         <v>2500</v>
       </c>
-      <c r="H5" s="71" t="n">
+      <c r="H5" s="75" t="n">
         <v>5000</v>
       </c>
-      <c r="I5" s="72" t="n">
+      <c r="I5" s="76" t="n">
         <v>45000</v>
       </c>
-      <c r="J5" s="68" t="inlineStr"/>
-      <c r="K5" s="68" t="inlineStr"/>
-      <c r="L5" s="68" t="inlineStr">
+      <c r="J5" s="72" t="inlineStr"/>
+      <c r="K5" s="72" t="inlineStr"/>
+      <c r="L5" s="72" t="inlineStr">
         <is>
           <t>Transferencia mensual</t>
         </is>
       </c>
-      <c r="M5" s="68" t="inlineStr">
+      <c r="M5" s="72" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="N5" s="68" t="inlineStr">
+      <c r="N5" s="72" t="inlineStr">
         <is>
           <t>Prestamo dic 2025. Capital $50K. Interes 5% mensual $2,500. Abono $5K capital el 29-abr-26. Saldo vivo $45K.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="73" t="inlineStr">
+      <c r="A10" s="77" t="inlineStr">
         <is>
           <t>TOTAL POR PAGAR</t>
         </is>
       </c>
-      <c r="C10" s="66" t="n">
+      <c r="C10" s="78" t="n">
         <v>90000</v>
       </c>
-      <c r="G10" s="74" t="n">
+      <c r="G10" s="79" t="n">
         <v>4100</v>
       </c>
-      <c r="H10" s="74" t="n">
+      <c r="H10" s="79" t="n">
         <v>5000</v>
       </c>
-      <c r="I10" s="75" t="n">
+      <c r="I10" s="80" t="n">
         <v>85000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="76" t="inlineStr">
+      <c r="A14" s="81" t="inlineStr">
         <is>
           <t>CREDITO ROTATIVO PROVEEDOR</t>
         </is>
@@ -3629,20 +3751,20 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="77" t="inlineStr">
+      <c r="A16" s="82" t="inlineStr">
         <is>
           <t>Olivar Andaluz S.L.</t>
         </is>
       </c>
-      <c r="B16" s="78" t="inlineStr">
+      <c r="B16" s="83" t="inlineStr">
         <is>
           <t>Cisterna 18 (OL180)</t>
         </is>
       </c>
-      <c r="C16" s="58" t="n">
+      <c r="C16" s="84" t="n">
         <v>58420.5</v>
       </c>
-      <c r="D16" s="78" t="inlineStr">
+      <c r="D16" s="83" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -3663,164 +3785,437 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C17"/>
+  <dimension ref="B2:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="79" t="inlineStr">
-        <is>
-          <t>KPIs (referencia tecnica)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="80" t="inlineStr">
-        <is>
-          <t>Total Ingresos</t>
-        </is>
-      </c>
-      <c r="C5" s="81">
+    <row r="2" ht="44" customHeight="1">
+      <c r="B2" s="85" t="inlineStr">
+        <is>
+          <t>KPIs OPERATIVOS  ·  OLIVAR DEL SUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Mes en curso · Mayo 2026  ·  Datos vivos: cualquier captura nueva recalcula esta vista</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>FLUJO NETO DEL PERIODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="86">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in")-SUMIFS(Transacciones!D:D,Transacciones!E:E,"out")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Ingresos cobrados − Gastos pagados</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>DESGLOSE DE INGRESOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>COBROS A CLIENTES</t>
+        </is>
+      </c>
+      <c r="D12" s="87" t="inlineStr">
+        <is>
+          <t>COBROS A CREDITO</t>
+        </is>
+      </c>
+      <c r="F12" s="87" t="inlineStr">
+        <is>
+          <t>RETORNO GANDOLAS</t>
+        </is>
+      </c>
+      <c r="H12" s="88" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="B13" s="89">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"cobro_cliente")</f>
+        <v/>
+      </c>
+      <c r="D13" s="89">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"cobro_credito")</f>
+        <v/>
+      </c>
+      <c r="F13" s="89">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"retorno_gandola")</f>
+        <v/>
+      </c>
+      <c r="H13" s="90">
         <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"in")</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="80" t="inlineStr">
-        <is>
-          <t>Total Gastos</t>
-        </is>
-      </c>
-      <c r="C6" s="81">
+    <row r="14" ht="16" customHeight="1">
+      <c r="B14" s="91" t="inlineStr">
+        <is>
+          <t>Categoria cobro_cliente</t>
+        </is>
+      </c>
+      <c r="D14" s="91" t="inlineStr">
+        <is>
+          <t>Categoria cobro_credito</t>
+        </is>
+      </c>
+      <c r="F14" s="91" t="inlineStr">
+        <is>
+          <t>Categoria retorno_gandola</t>
+        </is>
+      </c>
+      <c r="H14" s="92" t="inlineStr">
+        <is>
+          <t>Suma direccion in</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>DESGLOSE DE GASTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="93" t="inlineStr">
+        <is>
+          <t>PAGOS A PROVEEDORES</t>
+        </is>
+      </c>
+      <c r="D19" s="93" t="inlineStr">
+        <is>
+          <t>INTERES DE DEUDA</t>
+        </is>
+      </c>
+      <c r="F19" s="93" t="inlineStr">
+        <is>
+          <t>CAPITAL DE DEUDA</t>
+        </is>
+      </c>
+      <c r="H19" s="88" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="B20" s="94">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"pago_proveedor")</f>
+        <v/>
+      </c>
+      <c r="D20" s="94">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"pago_deuda_interes")</f>
+        <v/>
+      </c>
+      <c r="F20" s="94">
+        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"pago_deuda_capital")</f>
+        <v/>
+      </c>
+      <c r="H20" s="90">
         <f>SUMIFS(Transacciones!D:D,Transacciones!E:E,"out")</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="80" t="inlineStr">
-        <is>
-          <t>Pagos a Proveedores</t>
-        </is>
-      </c>
-      <c r="C7" s="81">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"pago_proveedor")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="80" t="inlineStr">
-        <is>
-          <t>Pagos Deuda Interes</t>
-        </is>
-      </c>
-      <c r="C8" s="81">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"pago_deuda_interes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="80" t="inlineStr">
-        <is>
-          <t>Pagos Deuda Capital</t>
-        </is>
-      </c>
-      <c r="C9" s="81">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"pago_deuda_capital")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="80" t="inlineStr">
-        <is>
-          <t>Cobros Clientes</t>
-        </is>
-      </c>
-      <c r="C10" s="81">
-        <f>SUMIFS(Transacciones!D:D,Transacciones!F:F,"cobro_cliente")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="80" t="inlineStr">
-        <is>
-          <t>Flujo Neto</t>
-        </is>
-      </c>
-      <c r="C11" s="81">
-        <f>C5-C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="80" t="inlineStr">
-        <is>
-          <t># Cobros</t>
-        </is>
-      </c>
-      <c r="C12" s="82">
+    <row r="21" ht="16" customHeight="1">
+      <c r="B21" s="95" t="inlineStr">
+        <is>
+          <t>Categoria pago_proveedor</t>
+        </is>
+      </c>
+      <c r="D21" s="95" t="inlineStr">
+        <is>
+          <t>Categoria pago_deuda_interes</t>
+        </is>
+      </c>
+      <c r="F21" s="95" t="inlineStr">
+        <is>
+          <t>Abonos a principal</t>
+        </is>
+      </c>
+      <c r="H21" s="92" t="inlineStr">
+        <is>
+          <t>Suma direccion out</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>OPERACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="96" t="inlineStr">
+        <is>
+          <t># COBROS RECIBIDOS</t>
+        </is>
+      </c>
+      <c r="D26" s="96" t="inlineStr">
+        <is>
+          <t># PAGOS REALIZADOS</t>
+        </is>
+      </c>
+      <c r="F26" s="96" t="inlineStr">
+        <is>
+          <t>TICKET PROMEDIO COBRO</t>
+        </is>
+      </c>
+      <c r="H26" s="96" t="inlineStr">
+        <is>
+          <t>TICKET PROMEDIO GASTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="B27" s="97">
         <f>COUNTIFS(Transacciones!E:E,"in")</f>
         <v/>
       </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="80" t="inlineStr">
-        <is>
-          <t># Pagos</t>
-        </is>
-      </c>
-      <c r="C13" s="82">
+      <c r="D27" s="97">
         <f>COUNTIFS(Transacciones!E:E,"out")</f>
         <v/>
       </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="80" t="inlineStr">
-        <is>
-          <t>Banco (calculado)</t>
-        </is>
-      </c>
-      <c r="C14" s="81">
+      <c r="F27" s="98">
+        <f>IFERROR(SUMIFS(Transacciones!D:D,Transacciones!E:E,"in")/COUNTIFS(Transacciones!E:E,"in"),0)</f>
+        <v/>
+      </c>
+      <c r="H27" s="98">
+        <f>IFERROR(SUMIFS(Transacciones!D:D,Transacciones!E:E,"out")/COUNTIFS(Transacciones!E:E,"out"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="B28" s="99" t="inlineStr">
+        <is>
+          <t>Capturas entrantes</t>
+        </is>
+      </c>
+      <c r="D28" s="99" t="inlineStr">
+        <is>
+          <t>Salidas de caja</t>
+        </is>
+      </c>
+      <c r="F28" s="99" t="inlineStr">
+        <is>
+          <t>Promedio por captura</t>
+        </is>
+      </c>
+      <c r="H28" s="99" t="inlineStr">
+        <is>
+          <t>Promedio salida</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="B31" s="26" t="inlineStr">
+        <is>
+          <t>POSICION DE EFECTIVO  (link Dashboard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="96" t="inlineStr">
+        <is>
+          <t>EFECTIVO EN BANCO</t>
+        </is>
+      </c>
+      <c r="D33" s="100" t="inlineStr">
+        <is>
+          <t>CAPITAL EN GANDOLAS</t>
+        </is>
+      </c>
+      <c r="F33" s="101" t="inlineStr">
+        <is>
+          <t>CUENTAS POR COBRAR</t>
+        </is>
+      </c>
+      <c r="H33" s="88" t="inlineStr">
+        <is>
+          <t>TOTAL TRAZADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="B34" s="102">
         <f>Dashboard!C12</f>
         <v/>
       </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="80" t="inlineStr">
-        <is>
-          <t>Gandolas (calculado)</t>
-        </is>
-      </c>
-      <c r="C15" s="81">
+      <c r="D34" s="103">
         <f>Dashboard!E12</f>
         <v/>
       </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="80" t="inlineStr">
-        <is>
-          <t>Por Cobrar (calculado)</t>
-        </is>
-      </c>
-      <c r="C16" s="81">
+      <c r="F34" s="104">
         <f>Dashboard!G12</f>
         <v/>
       </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="80" t="inlineStr">
-        <is>
-          <t>Total Trazado</t>
-        </is>
-      </c>
-      <c r="C17" s="81">
+      <c r="H34" s="90">
         <f>Dashboard!B8</f>
         <v/>
       </c>
     </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="B35" s="99" t="inlineStr">
+        <is>
+          <t>Saldo liquido</t>
+        </is>
+      </c>
+      <c r="D35" s="105" t="inlineStr">
+        <is>
+          <t>En transito</t>
+        </is>
+      </c>
+      <c r="F35" s="106" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H35" s="92" t="inlineStr">
+        <is>
+          <t>Suma 3 buckets</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="107" t="inlineStr">
+        <is>
+          <t>Convencion de colores (estandar finance / IB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="82" t="inlineStr">
+        <is>
+          <t>AZUL</t>
+        </is>
+      </c>
+      <c r="C39" s="108" t="inlineStr">
+        <is>
+          <t>input hardcodeado (saldo inicial, datos de transaccion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="42" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="C40" s="108" t="inlineStr">
+        <is>
+          <t>formula que opera sobre celdas de la misma pestaña</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="109" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="C41" s="108" t="inlineStr">
+        <is>
+          <t>formula que referencia OTRA pestaña (link cross-sheet)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="61">
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="H26:I26"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>